<commit_message>
Week 5 OF  IT Goverance Project
</commit_message>
<xml_diff>
--- a/IT Risk Register.xlsx
+++ b/IT Risk Register.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\salmo\Desktop\Tech\03 Projects\Enterprise Network Lab\03 Governance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C26F84-9A17-4649-9297-6F5AEB7CCE99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD1DC5F-B2D1-45BF-9F35-4202CBAC1695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{EE207035-1F51-4DCC-B353-2E8B956805B3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EE207035-1F51-4DCC-B353-2E8B956805B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Operational Risk Register" sheetId="1" r:id="rId1"/>
@@ -294,7 +294,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="191">
   <si>
     <t>Risk Title</t>
   </si>
@@ -719,9 +719,6 @@
     <t>Strategic</t>
   </si>
   <si>
-    <t>If the single inter-VLAN router fails while acting as the network gateway, the network becomes vulnerable to total internal connectivity loss resulting in operational disruption.</t>
-  </si>
-  <si>
     <t>If an access switch fails without redundancy, connected departments become vulnerable to complete network isolation resulting in service disruption.</t>
   </si>
   <si>
@@ -755,9 +752,6 @@
     <t>If infrastructure documentation is missing or incomplete, recovery operations become vulnerable to delays resulting in prolonged outages.</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>IT Infrastructure Manager</t>
   </si>
   <si>
@@ -843,12 +837,45 @@
   </si>
   <si>
     <t>Design and Implement an In-House Network Monitoring Capability</t>
+  </si>
+  <si>
+    <t>Centralized, auditable change management system</t>
+  </si>
+  <si>
+    <t>If the single core router fails while providing inter-VLAN routing, inter-campus connectivity, and DHCP relay services, the network risks widespread cross-site communication failure and loss of critical services, resulting in operational disruption.</t>
+  </si>
+  <si>
+    <t>Manual failover using router substitution for Campus A recovery and degraded standalone operation for Campus B including manual IP configuration and local service provisioning</t>
+  </si>
+  <si>
+    <t>Maintain operational continuity during router failure by enabling Campus B standalone operation, pre-staging critical data locally, and supporting rapid recovery of Campus A through hardware reallocation.</t>
+  </si>
+  <si>
+    <t>Eliminate single points of failure by implementing redundant routing and dual-site service capability with replicated infrastructure.</t>
+  </si>
+  <si>
+    <t>Implement and validate manual failover procedures including router substitution for Campus A recovery and degraded standalone operation for Campus B with manual IP configuration and local service activation</t>
+  </si>
+  <si>
+    <t>Change Management Policy v1.0</t>
+  </si>
+  <si>
+    <t>Implement Change Management Procedure v1.0 (aligned to Change Management Policy v1.0)</t>
+  </si>
+  <si>
+    <t>Achieved – Formal change management process established</t>
+  </si>
+  <si>
+    <t>Develop a centralized application to automate and improve implementation of the change control policy</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -900,7 +927,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -910,6 +937,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1100,7 +1139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1138,23 +1177,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1162,10 +1189,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1188,6 +1242,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1571,86 +1631,86 @@
     <col min="11" max="11" width="9" style="4" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="55.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="67.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="59.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="46.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="48.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="30" style="4" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="33.85546875" style="4" customWidth="1"/>
     <col min="20" max="20" width="51.140625" style="5" customWidth="1"/>
-    <col min="21" max="21" width="16.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.28515625" style="20" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.42578125" style="21" bestFit="1" customWidth="1"/>
     <col min="24" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="F1" s="27" t="s">
+      <c r="F1" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="28"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="27" t="s">
+      <c r="G1" s="33"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="28"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="25" t="s">
+      <c r="J1" s="33"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="25" t="s">
+      <c r="M1" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="25" t="s">
+      <c r="N1" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="25" t="s">
+      <c r="O1" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="P1" s="25" t="s">
+      <c r="P1" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="Q1" s="25" t="s">
+      <c r="Q1" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="R1" s="25" t="s">
+      <c r="R1" s="30" t="s">
         <v>119</v>
       </c>
-      <c r="S1" s="25" t="s">
+      <c r="S1" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="T1" s="27" t="s">
+      <c r="T1" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="U1" s="29"/>
-      <c r="V1" s="21" t="s">
+      <c r="U1" s="34"/>
+      <c r="V1" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="W1" s="21" t="s">
+      <c r="W1" s="26" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:23" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="22"/>
+      <c r="A2" s="31"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="25"/>
       <c r="F2" s="9" t="s">
         <v>1</v>
       </c>
@@ -1669,100 +1729,100 @@
       <c r="K2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="26"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="31"/>
+      <c r="R2" s="31"/>
+      <c r="S2" s="31"/>
       <c r="T2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="U2" s="11" t="s">
+      <c r="U2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
+      <c r="V2" s="25"/>
+      <c r="W2" s="27"/>
     </row>
     <row r="3" spans="1:23" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="A3" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C3" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="F3" s="2">
+      <c r="E3" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="F3" s="13">
         <v>4</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="13">
         <v>4</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="13">
         <f t="shared" ref="H3:H14" si="0">F3*G3</f>
         <v>16</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="13">
         <v>4</v>
       </c>
-      <c r="J3" s="2">
-        <v>2</v>
-      </c>
-      <c r="K3" s="2">
+      <c r="J3" s="13">
+        <v>4</v>
+      </c>
+      <c r="K3" s="13">
         <f t="shared" ref="K3:K14" si="1">I3*J3</f>
-        <v>8</v>
-      </c>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2">
+        <v>16</v>
+      </c>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13">
         <v>1</v>
       </c>
-      <c r="N3" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="O3" s="2" t="s">
+      <c r="N3" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="P3" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="T3" s="3" t="s">
+      <c r="O3" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="U3" s="13">
-        <v>46419</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="W3" s="13">
-        <v>46113</v>
+      <c r="P3" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q3" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="R3" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="S3" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="T3" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="U3" s="35">
+        <v>46132</v>
+      </c>
+      <c r="V3" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="W3" s="17">
+        <v>46133</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>137</v>
@@ -1771,7 +1831,7 @@
         <v>139</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F4" s="6">
         <v>4</v>
@@ -1784,120 +1844,136 @@
         <v>16</v>
       </c>
       <c r="I4" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J4" s="6">
         <v>4</v>
       </c>
       <c r="K4" s="6">
         <f t="shared" si="1"/>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="L4" s="6"/>
       <c r="M4" s="6">
         <v>2</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="P4" s="6" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="P4" s="36" t="s">
+        <v>189</v>
       </c>
       <c r="Q4" s="6" t="s">
         <v>181</v>
       </c>
       <c r="R4" s="6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="S4" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="T4" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="U4" s="17">
+        <v>46147</v>
+      </c>
+      <c r="V4" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="T4" s="7" t="s">
+      <c r="W4" s="18">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="U4" s="14">
-        <v>46120</v>
-      </c>
-      <c r="V4" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="W4" s="14">
-        <v>46120</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="F5" s="15">
-        <v>4</v>
-      </c>
-      <c r="G5" s="15">
-        <v>4</v>
-      </c>
-      <c r="H5" s="15">
+      <c r="F5" s="2">
+        <v>3</v>
+      </c>
+      <c r="G5" s="2">
+        <v>5</v>
+      </c>
+      <c r="H5" s="2">
         <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="I5" s="15">
-        <v>4</v>
-      </c>
-      <c r="J5" s="15">
-        <v>4</v>
-      </c>
-      <c r="K5" s="15">
+        <v>15</v>
+      </c>
+      <c r="I5" s="2">
+        <v>3</v>
+      </c>
+      <c r="J5" s="2">
+        <v>5</v>
+      </c>
+      <c r="K5" s="2">
         <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15">
+        <v>15</v>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2">
         <v>3</v>
       </c>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
-      <c r="S5" s="15"/>
-      <c r="T5" s="16"/>
-      <c r="U5" s="17"/>
-      <c r="V5" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="W5" s="17">
-        <v>46089</v>
+      <c r="N5" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="P5" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="T5" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="U5" s="19">
+        <v>46140</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="W5" s="19">
+        <v>46133</v>
       </c>
     </row>
     <row r="6" spans="1:23" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>139</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="F6" s="4">
         <v>3</v>
@@ -1922,75 +1998,74 @@
       <c r="M6" s="4">
         <v>4</v>
       </c>
-      <c r="U6" s="18"/>
       <c r="V6" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="W6" s="18">
+        <v>154</v>
+      </c>
+      <c r="W6" s="20">
         <v>46089</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="A7" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="F7" s="2">
+      <c r="E7" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="F7" s="13">
         <v>3</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="13">
+        <v>4</v>
+      </c>
+      <c r="H7" s="13">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="I7" s="13">
+        <v>3</v>
+      </c>
+      <c r="J7" s="13">
+        <v>4</v>
+      </c>
+      <c r="K7" s="13">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13">
         <v>5</v>
       </c>
-      <c r="H7" s="2">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="I7" s="2">
-        <v>3</v>
-      </c>
-      <c r="J7" s="2">
-        <v>5</v>
-      </c>
-      <c r="K7" s="2">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2">
-        <v>5</v>
-      </c>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="13"/>
-      <c r="V7" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="W7" s="13">
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="13"/>
+      <c r="Q7" s="13"/>
+      <c r="R7" s="13"/>
+      <c r="S7" s="13"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="17"/>
+      <c r="V7" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="W7" s="17">
         <v>46089</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>136</v>
@@ -1999,7 +2074,7 @@
         <v>139</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="F8" s="6">
         <v>3</v>
@@ -2032,84 +2107,84 @@
       <c r="R8" s="6"/>
       <c r="S8" s="6"/>
       <c r="T8" s="7"/>
-      <c r="U8" s="14"/>
+      <c r="U8" s="18"/>
       <c r="V8" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="W8" s="14">
+        <v>154</v>
+      </c>
+      <c r="W8" s="18">
         <v>46089</v>
       </c>
     </row>
     <row r="9" spans="1:23" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="C9" s="15" t="s">
+      <c r="A9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="2">
         <v>3</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="2">
         <v>4</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="I9" s="15">
+      <c r="I9" s="2">
         <v>3</v>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="2">
         <v>4</v>
       </c>
-      <c r="K9" s="15">
+      <c r="K9" s="2">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="L9" s="15"/>
-      <c r="M9" s="15">
+      <c r="L9" s="2"/>
+      <c r="M9" s="2">
         <v>7</v>
       </c>
-      <c r="N9" s="15"/>
-      <c r="O9" s="15"/>
-      <c r="P9" s="15"/>
-      <c r="Q9" s="15"/>
-      <c r="R9" s="15"/>
-      <c r="S9" s="15"/>
-      <c r="T9" s="16"/>
-      <c r="U9" s="17"/>
-      <c r="V9" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="W9" s="17">
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="2"/>
+      <c r="T9" s="3"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="W9" s="19">
         <v>46089</v>
       </c>
     </row>
     <row r="10" spans="1:23" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>136</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F10" s="4">
         <v>3</v>
@@ -2134,232 +2209,232 @@
       <c r="M10" s="4">
         <v>8</v>
       </c>
-      <c r="U10" s="18"/>
       <c r="V10" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="W10" s="18">
+        <v>154</v>
+      </c>
+      <c r="W10" s="20">
         <v>46089</v>
       </c>
     </row>
     <row r="11" spans="1:23" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="F11" s="2">
+      <c r="A11" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="F11" s="13">
         <v>3</v>
       </c>
-      <c r="G11" s="2">
-        <v>4</v>
-      </c>
-      <c r="H11" s="2">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="I11" s="2">
+      <c r="G11" s="13">
         <v>3</v>
       </c>
-      <c r="J11" s="2">
-        <v>4</v>
-      </c>
-      <c r="K11" s="2">
-        <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2">
-        <v>9</v>
-      </c>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-      <c r="T11" s="3"/>
-      <c r="U11" s="13"/>
-      <c r="V11" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="W11" s="13">
-        <v>46089</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="F12" s="6">
-        <v>3</v>
-      </c>
-      <c r="G12" s="6">
-        <v>3</v>
-      </c>
-      <c r="H12" s="6">
+      <c r="H11" s="13">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I12" s="6">
+      <c r="I11" s="13">
         <v>3</v>
       </c>
-      <c r="J12" s="6">
+      <c r="J11" s="13">
         <v>3</v>
       </c>
-      <c r="K12" s="6">
+      <c r="K11" s="13">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6">
-        <v>10</v>
-      </c>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
-      <c r="T12" s="7"/>
-      <c r="U12" s="14"/>
-      <c r="V12" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="W12" s="14">
+      <c r="L11" s="13"/>
+      <c r="M11" s="13">
+        <v>9</v>
+      </c>
+      <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="13"/>
+      <c r="Q11" s="13"/>
+      <c r="R11" s="13"/>
+      <c r="S11" s="13"/>
+      <c r="T11" s="14"/>
+      <c r="U11" s="17"/>
+      <c r="V11" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="W11" s="17">
         <v>46089</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="12" spans="1:23" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D12" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="F13" s="2">
+      <c r="E12" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="F12" s="4">
         <v>3</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G12" s="4">
         <v>3</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H12" s="4">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I12" s="4">
         <v>3</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J12" s="4">
         <v>3</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K12" s="4">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2">
-        <v>11</v>
-      </c>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
-      <c r="T13" s="3"/>
-      <c r="U13" s="13"/>
-      <c r="V13" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="W13" s="13">
+      <c r="M12" s="4">
+        <v>10</v>
+      </c>
+      <c r="V12" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="W12" s="20">
         <v>46089</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+    <row r="13" spans="1:23" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B13" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C13" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D13" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="E14" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="F14" s="6">
+      <c r="E13" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="F13" s="13">
         <v>3</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G13" s="13">
         <v>3</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H13" s="13">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I14" s="6">
+      <c r="I13" s="13">
         <v>3</v>
       </c>
-      <c r="J14" s="6">
+      <c r="J13" s="13">
         <v>3</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K13" s="13">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6" t="s">
+      <c r="L13" s="13"/>
+      <c r="M13" s="13"/>
+      <c r="N13" s="13"/>
+      <c r="O13" s="13"/>
+      <c r="P13" s="13"/>
+      <c r="Q13" s="13"/>
+      <c r="R13" s="13"/>
+      <c r="S13" s="13"/>
+      <c r="T13" s="14"/>
+      <c r="U13" s="17"/>
+      <c r="V13" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="W13" s="17">
+        <v>46089</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F14" s="4">
+        <v>4</v>
+      </c>
+      <c r="G14" s="4">
+        <v>4</v>
+      </c>
+      <c r="H14" s="4">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="I14" s="4">
+        <v>4</v>
+      </c>
+      <c r="J14" s="4">
+        <v>2</v>
+      </c>
+      <c r="K14" s="4">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="R14" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="N14" s="6"/>
-      <c r="O14" s="6"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="6"/>
-      <c r="R14" s="6"/>
-      <c r="S14" s="6"/>
-      <c r="T14" s="7"/>
-      <c r="U14" s="14"/>
-      <c r="V14" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="W14" s="14">
-        <v>46089</v>
+      <c r="S14" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="T14" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="U14" s="20">
+        <v>46419</v>
+      </c>
+      <c r="V14" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="W14" s="20">
+        <v>46113</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -2385,9 +2460,9 @@
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
       <c r="T15" s="3"/>
-      <c r="U15" s="2"/>
+      <c r="U15" s="19"/>
       <c r="V15" s="2"/>
-      <c r="W15" s="2"/>
+      <c r="W15" s="19"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
@@ -2412,9 +2487,9 @@
       <c r="R16" s="6"/>
       <c r="S16" s="6"/>
       <c r="T16" s="7"/>
-      <c r="U16" s="6"/>
+      <c r="U16" s="18"/>
       <c r="V16" s="6"/>
-      <c r="W16" s="6"/>
+      <c r="W16" s="18"/>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
@@ -2439,9 +2514,9 @@
       <c r="R17" s="2"/>
       <c r="S17" s="2"/>
       <c r="T17" s="3"/>
-      <c r="U17" s="2"/>
+      <c r="U17" s="19"/>
       <c r="V17" s="2"/>
-      <c r="W17" s="2"/>
+      <c r="W17" s="19"/>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
@@ -2466,9 +2541,9 @@
       <c r="R18" s="6"/>
       <c r="S18" s="6"/>
       <c r="T18" s="7"/>
-      <c r="U18" s="6"/>
+      <c r="U18" s="18"/>
       <c r="V18" s="6"/>
-      <c r="W18" s="6"/>
+      <c r="W18" s="18"/>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
@@ -2493,9 +2568,9 @@
       <c r="R19" s="2"/>
       <c r="S19" s="2"/>
       <c r="T19" s="3"/>
-      <c r="U19" s="2"/>
+      <c r="U19" s="19"/>
       <c r="V19" s="2"/>
-      <c r="W19" s="2"/>
+      <c r="W19" s="19"/>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
@@ -2520,9 +2595,9 @@
       <c r="R20" s="6"/>
       <c r="S20" s="6"/>
       <c r="T20" s="7"/>
-      <c r="U20" s="6"/>
+      <c r="U20" s="18"/>
       <c r="V20" s="6"/>
-      <c r="W20" s="6"/>
+      <c r="W20" s="18"/>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
@@ -2547,9 +2622,9 @@
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
       <c r="T21" s="3"/>
-      <c r="U21" s="2"/>
+      <c r="U21" s="19"/>
       <c r="V21" s="2"/>
-      <c r="W21" s="2"/>
+      <c r="W21" s="19"/>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
@@ -2574,9 +2649,9 @@
       <c r="R22" s="6"/>
       <c r="S22" s="6"/>
       <c r="T22" s="7"/>
-      <c r="U22" s="6"/>
+      <c r="U22" s="18"/>
       <c r="V22" s="6"/>
-      <c r="W22" s="6"/>
+      <c r="W22" s="18"/>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
@@ -2601,9 +2676,9 @@
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="3"/>
-      <c r="U23" s="2"/>
+      <c r="U23" s="19"/>
       <c r="V23" s="2"/>
-      <c r="W23" s="2"/>
+      <c r="W23" s="19"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
@@ -2628,9 +2703,9 @@
       <c r="R24" s="6"/>
       <c r="S24" s="6"/>
       <c r="T24" s="7"/>
-      <c r="U24" s="6"/>
+      <c r="U24" s="18"/>
       <c r="V24" s="6"/>
-      <c r="W24" s="6"/>
+      <c r="W24" s="18"/>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
@@ -2655,9 +2730,9 @@
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
       <c r="T25" s="3"/>
-      <c r="U25" s="2"/>
+      <c r="U25" s="19"/>
       <c r="V25" s="2"/>
-      <c r="W25" s="2"/>
+      <c r="W25" s="19"/>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
@@ -2682,9 +2757,9 @@
       <c r="R26" s="6"/>
       <c r="S26" s="6"/>
       <c r="T26" s="7"/>
-      <c r="U26" s="6"/>
+      <c r="U26" s="18"/>
       <c r="V26" s="6"/>
-      <c r="W26" s="6"/>
+      <c r="W26" s="18"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
@@ -2709,9 +2784,9 @@
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
       <c r="T27" s="3"/>
-      <c r="U27" s="2"/>
+      <c r="U27" s="19"/>
       <c r="V27" s="2"/>
-      <c r="W27" s="2"/>
+      <c r="W27" s="19"/>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
@@ -2736,9 +2811,9 @@
       <c r="R28" s="6"/>
       <c r="S28" s="6"/>
       <c r="T28" s="7"/>
-      <c r="U28" s="6"/>
+      <c r="U28" s="18"/>
       <c r="V28" s="6"/>
-      <c r="W28" s="6"/>
+      <c r="W28" s="18"/>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
@@ -2763,9 +2838,9 @@
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
       <c r="T29" s="3"/>
-      <c r="U29" s="2"/>
+      <c r="U29" s="19"/>
       <c r="V29" s="2"/>
-      <c r="W29" s="2"/>
+      <c r="W29" s="19"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
@@ -2790,9 +2865,9 @@
       <c r="R30" s="6"/>
       <c r="S30" s="6"/>
       <c r="T30" s="7"/>
-      <c r="U30" s="6"/>
+      <c r="U30" s="18"/>
       <c r="V30" s="6"/>
-      <c r="W30" s="6"/>
+      <c r="W30" s="18"/>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
@@ -2817,9 +2892,9 @@
       <c r="R31" s="2"/>
       <c r="S31" s="2"/>
       <c r="T31" s="3"/>
-      <c r="U31" s="2"/>
+      <c r="U31" s="19"/>
       <c r="V31" s="2"/>
-      <c r="W31" s="2"/>
+      <c r="W31" s="19"/>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
@@ -2844,9 +2919,9 @@
       <c r="R32" s="6"/>
       <c r="S32" s="6"/>
       <c r="T32" s="7"/>
-      <c r="U32" s="6"/>
+      <c r="U32" s="18"/>
       <c r="V32" s="6"/>
-      <c r="W32" s="6"/>
+      <c r="W32" s="18"/>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
@@ -2871,9 +2946,9 @@
       <c r="R33" s="2"/>
       <c r="S33" s="2"/>
       <c r="T33" s="3"/>
-      <c r="U33" s="2"/>
+      <c r="U33" s="19"/>
       <c r="V33" s="2"/>
-      <c r="W33" s="2"/>
+      <c r="W33" s="19"/>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
@@ -2898,9 +2973,9 @@
       <c r="R34" s="6"/>
       <c r="S34" s="6"/>
       <c r="T34" s="7"/>
-      <c r="U34" s="6"/>
+      <c r="U34" s="18"/>
       <c r="V34" s="6"/>
-      <c r="W34" s="6"/>
+      <c r="W34" s="18"/>
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
@@ -2925,9 +3000,9 @@
       <c r="R35" s="2"/>
       <c r="S35" s="2"/>
       <c r="T35" s="3"/>
-      <c r="U35" s="2"/>
+      <c r="U35" s="19"/>
       <c r="V35" s="2"/>
-      <c r="W35" s="2"/>
+      <c r="W35" s="19"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
@@ -2952,9 +3027,9 @@
       <c r="R36" s="6"/>
       <c r="S36" s="6"/>
       <c r="T36" s="7"/>
-      <c r="U36" s="6"/>
+      <c r="U36" s="18"/>
       <c r="V36" s="6"/>
-      <c r="W36" s="6"/>
+      <c r="W36" s="18"/>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
@@ -2979,9 +3054,9 @@
       <c r="R37" s="2"/>
       <c r="S37" s="2"/>
       <c r="T37" s="3"/>
-      <c r="U37" s="2"/>
+      <c r="U37" s="19"/>
       <c r="V37" s="2"/>
-      <c r="W37" s="2"/>
+      <c r="W37" s="19"/>
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
@@ -3006,9 +3081,9 @@
       <c r="R38" s="6"/>
       <c r="S38" s="6"/>
       <c r="T38" s="7"/>
-      <c r="U38" s="6"/>
+      <c r="U38" s="18"/>
       <c r="V38" s="6"/>
-      <c r="W38" s="6"/>
+      <c r="W38" s="18"/>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
@@ -3033,9 +3108,9 @@
       <c r="R39" s="2"/>
       <c r="S39" s="2"/>
       <c r="T39" s="3"/>
-      <c r="U39" s="2"/>
+      <c r="U39" s="19"/>
       <c r="V39" s="2"/>
-      <c r="W39" s="2"/>
+      <c r="W39" s="19"/>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
@@ -3060,9 +3135,9 @@
       <c r="R40" s="6"/>
       <c r="S40" s="6"/>
       <c r="T40" s="7"/>
-      <c r="U40" s="6"/>
+      <c r="U40" s="18"/>
       <c r="V40" s="6"/>
-      <c r="W40" s="6"/>
+      <c r="W40" s="18"/>
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
@@ -3087,9 +3162,9 @@
       <c r="R41" s="2"/>
       <c r="S41" s="2"/>
       <c r="T41" s="3"/>
-      <c r="U41" s="2"/>
+      <c r="U41" s="19"/>
       <c r="V41" s="2"/>
-      <c r="W41" s="2"/>
+      <c r="W41" s="19"/>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
@@ -3114,9 +3189,9 @@
       <c r="R42" s="6"/>
       <c r="S42" s="6"/>
       <c r="T42" s="7"/>
-      <c r="U42" s="6"/>
+      <c r="U42" s="18"/>
       <c r="V42" s="6"/>
-      <c r="W42" s="6"/>
+      <c r="W42" s="18"/>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
@@ -3141,9 +3216,9 @@
       <c r="R43" s="2"/>
       <c r="S43" s="2"/>
       <c r="T43" s="3"/>
-      <c r="U43" s="2"/>
+      <c r="U43" s="19"/>
       <c r="V43" s="2"/>
-      <c r="W43" s="2"/>
+      <c r="W43" s="19"/>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
@@ -3168,9 +3243,9 @@
       <c r="R44" s="6"/>
       <c r="S44" s="6"/>
       <c r="T44" s="7"/>
-      <c r="U44" s="6"/>
+      <c r="U44" s="18"/>
       <c r="V44" s="6"/>
-      <c r="W44" s="6"/>
+      <c r="W44" s="18"/>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
@@ -3195,9 +3270,9 @@
       <c r="R45" s="2"/>
       <c r="S45" s="2"/>
       <c r="T45" s="3"/>
-      <c r="U45" s="2"/>
+      <c r="U45" s="19"/>
       <c r="V45" s="2"/>
-      <c r="W45" s="2"/>
+      <c r="W45" s="19"/>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
@@ -3222,9 +3297,9 @@
       <c r="R46" s="6"/>
       <c r="S46" s="6"/>
       <c r="T46" s="7"/>
-      <c r="U46" s="6"/>
+      <c r="U46" s="18"/>
       <c r="V46" s="6"/>
-      <c r="W46" s="6"/>
+      <c r="W46" s="18"/>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
@@ -3249,9 +3324,9 @@
       <c r="R47" s="2"/>
       <c r="S47" s="2"/>
       <c r="T47" s="3"/>
-      <c r="U47" s="2"/>
+      <c r="U47" s="19"/>
       <c r="V47" s="2"/>
-      <c r="W47" s="2"/>
+      <c r="W47" s="19"/>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
@@ -3276,9 +3351,9 @@
       <c r="R48" s="6"/>
       <c r="S48" s="6"/>
       <c r="T48" s="7"/>
-      <c r="U48" s="6"/>
+      <c r="U48" s="18"/>
       <c r="V48" s="6"/>
-      <c r="W48" s="6"/>
+      <c r="W48" s="18"/>
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
@@ -3303,9 +3378,9 @@
       <c r="R49" s="2"/>
       <c r="S49" s="2"/>
       <c r="T49" s="3"/>
-      <c r="U49" s="2"/>
+      <c r="U49" s="19"/>
       <c r="V49" s="2"/>
-      <c r="W49" s="2"/>
+      <c r="W49" s="19"/>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
@@ -3330,9 +3405,9 @@
       <c r="R50" s="6"/>
       <c r="S50" s="6"/>
       <c r="T50" s="7"/>
-      <c r="U50" s="6"/>
+      <c r="U50" s="18"/>
       <c r="V50" s="6"/>
-      <c r="W50" s="6"/>
+      <c r="W50" s="18"/>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
@@ -3357,9 +3432,9 @@
       <c r="R51" s="2"/>
       <c r="S51" s="2"/>
       <c r="T51" s="3"/>
-      <c r="U51" s="2"/>
+      <c r="U51" s="19"/>
       <c r="V51" s="2"/>
-      <c r="W51" s="2"/>
+      <c r="W51" s="19"/>
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
@@ -3384,9 +3459,9 @@
       <c r="R52" s="6"/>
       <c r="S52" s="6"/>
       <c r="T52" s="7"/>
-      <c r="U52" s="6"/>
+      <c r="U52" s="18"/>
       <c r="V52" s="6"/>
-      <c r="W52" s="6"/>
+      <c r="W52" s="18"/>
     </row>
     <row r="53" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
@@ -3411,9 +3486,9 @@
       <c r="R53" s="2"/>
       <c r="S53" s="2"/>
       <c r="T53" s="3"/>
-      <c r="U53" s="2"/>
+      <c r="U53" s="19"/>
       <c r="V53" s="2"/>
-      <c r="W53" s="2"/>
+      <c r="W53" s="19"/>
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
@@ -3438,9 +3513,9 @@
       <c r="R54" s="6"/>
       <c r="S54" s="6"/>
       <c r="T54" s="7"/>
-      <c r="U54" s="6"/>
+      <c r="U54" s="18"/>
       <c r="V54" s="6"/>
-      <c r="W54" s="6"/>
+      <c r="W54" s="18"/>
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
@@ -3465,9 +3540,9 @@
       <c r="R55" s="2"/>
       <c r="S55" s="2"/>
       <c r="T55" s="3"/>
-      <c r="U55" s="2"/>
+      <c r="U55" s="19"/>
       <c r="V55" s="2"/>
-      <c r="W55" s="2"/>
+      <c r="W55" s="19"/>
     </row>
     <row r="56" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
@@ -3492,9 +3567,9 @@
       <c r="R56" s="6"/>
       <c r="S56" s="6"/>
       <c r="T56" s="7"/>
-      <c r="U56" s="6"/>
+      <c r="U56" s="18"/>
       <c r="V56" s="6"/>
-      <c r="W56" s="6"/>
+      <c r="W56" s="18"/>
     </row>
     <row r="57" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
@@ -3519,9 +3594,9 @@
       <c r="R57" s="2"/>
       <c r="S57" s="2"/>
       <c r="T57" s="3"/>
-      <c r="U57" s="2"/>
+      <c r="U57" s="19"/>
       <c r="V57" s="2"/>
-      <c r="W57" s="2"/>
+      <c r="W57" s="19"/>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
@@ -3546,9 +3621,9 @@
       <c r="R58" s="6"/>
       <c r="S58" s="6"/>
       <c r="T58" s="7"/>
-      <c r="U58" s="6"/>
+      <c r="U58" s="18"/>
       <c r="V58" s="6"/>
-      <c r="W58" s="6"/>
+      <c r="W58" s="18"/>
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
@@ -3573,9 +3648,9 @@
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
       <c r="T59" s="3"/>
-      <c r="U59" s="2"/>
+      <c r="U59" s="19"/>
       <c r="V59" s="2"/>
-      <c r="W59" s="2"/>
+      <c r="W59" s="19"/>
     </row>
     <row r="60" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
@@ -3600,9 +3675,9 @@
       <c r="R60" s="6"/>
       <c r="S60" s="6"/>
       <c r="T60" s="7"/>
-      <c r="U60" s="6"/>
+      <c r="U60" s="18"/>
       <c r="V60" s="6"/>
-      <c r="W60" s="6"/>
+      <c r="W60" s="18"/>
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
@@ -3627,9 +3702,9 @@
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
       <c r="T61" s="3"/>
-      <c r="U61" s="2"/>
+      <c r="U61" s="19"/>
       <c r="V61" s="2"/>
-      <c r="W61" s="2"/>
+      <c r="W61" s="19"/>
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
@@ -3654,9 +3729,9 @@
       <c r="R62" s="6"/>
       <c r="S62" s="6"/>
       <c r="T62" s="7"/>
-      <c r="U62" s="6"/>
+      <c r="U62" s="18"/>
       <c r="V62" s="6"/>
-      <c r="W62" s="6"/>
+      <c r="W62" s="18"/>
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
@@ -3681,9 +3756,9 @@
       <c r="R63" s="2"/>
       <c r="S63" s="2"/>
       <c r="T63" s="3"/>
-      <c r="U63" s="2"/>
+      <c r="U63" s="19"/>
       <c r="V63" s="2"/>
-      <c r="W63" s="2"/>
+      <c r="W63" s="19"/>
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
@@ -3708,9 +3783,9 @@
       <c r="R64" s="6"/>
       <c r="S64" s="6"/>
       <c r="T64" s="7"/>
-      <c r="U64" s="6"/>
+      <c r="U64" s="18"/>
       <c r="V64" s="6"/>
-      <c r="W64" s="6"/>
+      <c r="W64" s="18"/>
     </row>
     <row r="65" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
@@ -3735,9 +3810,9 @@
       <c r="R65" s="2"/>
       <c r="S65" s="2"/>
       <c r="T65" s="3"/>
-      <c r="U65" s="2"/>
+      <c r="U65" s="19"/>
       <c r="V65" s="2"/>
-      <c r="W65" s="2"/>
+      <c r="W65" s="19"/>
     </row>
     <row r="66" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
@@ -3762,9 +3837,9 @@
       <c r="R66" s="6"/>
       <c r="S66" s="6"/>
       <c r="T66" s="7"/>
-      <c r="U66" s="6"/>
+      <c r="U66" s="18"/>
       <c r="V66" s="6"/>
-      <c r="W66" s="6"/>
+      <c r="W66" s="18"/>
     </row>
     <row r="67" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
@@ -3789,9 +3864,9 @@
       <c r="R67" s="2"/>
       <c r="S67" s="2"/>
       <c r="T67" s="3"/>
-      <c r="U67" s="2"/>
+      <c r="U67" s="19"/>
       <c r="V67" s="2"/>
-      <c r="W67" s="2"/>
+      <c r="W67" s="19"/>
     </row>
     <row r="68" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
@@ -3816,9 +3891,9 @@
       <c r="R68" s="6"/>
       <c r="S68" s="6"/>
       <c r="T68" s="7"/>
-      <c r="U68" s="6"/>
+      <c r="U68" s="18"/>
       <c r="V68" s="6"/>
-      <c r="W68" s="6"/>
+      <c r="W68" s="18"/>
     </row>
     <row r="69" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
@@ -3843,9 +3918,9 @@
       <c r="R69" s="2"/>
       <c r="S69" s="2"/>
       <c r="T69" s="3"/>
-      <c r="U69" s="2"/>
+      <c r="U69" s="19"/>
       <c r="V69" s="2"/>
-      <c r="W69" s="2"/>
+      <c r="W69" s="19"/>
     </row>
     <row r="70" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
@@ -3870,9 +3945,9 @@
       <c r="R70" s="6"/>
       <c r="S70" s="6"/>
       <c r="T70" s="7"/>
-      <c r="U70" s="6"/>
+      <c r="U70" s="18"/>
       <c r="V70" s="6"/>
-      <c r="W70" s="6"/>
+      <c r="W70" s="18"/>
     </row>
     <row r="71" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
@@ -3897,9 +3972,9 @@
       <c r="R71" s="2"/>
       <c r="S71" s="2"/>
       <c r="T71" s="3"/>
-      <c r="U71" s="2"/>
+      <c r="U71" s="19"/>
       <c r="V71" s="2"/>
-      <c r="W71" s="2"/>
+      <c r="W71" s="19"/>
     </row>
     <row r="72" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
@@ -3924,9 +3999,9 @@
       <c r="R72" s="6"/>
       <c r="S72" s="6"/>
       <c r="T72" s="7"/>
-      <c r="U72" s="6"/>
+      <c r="U72" s="18"/>
       <c r="V72" s="6"/>
-      <c r="W72" s="6"/>
+      <c r="W72" s="18"/>
     </row>
     <row r="73" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
@@ -3951,9 +4026,9 @@
       <c r="R73" s="2"/>
       <c r="S73" s="2"/>
       <c r="T73" s="3"/>
-      <c r="U73" s="2"/>
+      <c r="U73" s="19"/>
       <c r="V73" s="2"/>
-      <c r="W73" s="2"/>
+      <c r="W73" s="19"/>
     </row>
     <row r="74" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
@@ -3978,9 +4053,9 @@
       <c r="R74" s="6"/>
       <c r="S74" s="6"/>
       <c r="T74" s="7"/>
-      <c r="U74" s="6"/>
+      <c r="U74" s="18"/>
       <c r="V74" s="6"/>
-      <c r="W74" s="6"/>
+      <c r="W74" s="18"/>
     </row>
     <row r="75" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
@@ -4005,9 +4080,9 @@
       <c r="R75" s="2"/>
       <c r="S75" s="2"/>
       <c r="T75" s="3"/>
-      <c r="U75" s="2"/>
+      <c r="U75" s="19"/>
       <c r="V75" s="2"/>
-      <c r="W75" s="2"/>
+      <c r="W75" s="19"/>
     </row>
     <row r="76" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
@@ -4032,9 +4107,9 @@
       <c r="R76" s="6"/>
       <c r="S76" s="6"/>
       <c r="T76" s="7"/>
-      <c r="U76" s="6"/>
+      <c r="U76" s="18"/>
       <c r="V76" s="6"/>
-      <c r="W76" s="6"/>
+      <c r="W76" s="18"/>
     </row>
     <row r="77" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
@@ -4059,9 +4134,9 @@
       <c r="R77" s="2"/>
       <c r="S77" s="2"/>
       <c r="T77" s="3"/>
-      <c r="U77" s="2"/>
+      <c r="U77" s="19"/>
       <c r="V77" s="2"/>
-      <c r="W77" s="2"/>
+      <c r="W77" s="19"/>
     </row>
     <row r="78" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
@@ -4086,9 +4161,9 @@
       <c r="R78" s="6"/>
       <c r="S78" s="6"/>
       <c r="T78" s="7"/>
-      <c r="U78" s="6"/>
+      <c r="U78" s="18"/>
       <c r="V78" s="6"/>
-      <c r="W78" s="6"/>
+      <c r="W78" s="18"/>
     </row>
     <row r="79" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
@@ -4113,9 +4188,9 @@
       <c r="R79" s="2"/>
       <c r="S79" s="2"/>
       <c r="T79" s="3"/>
-      <c r="U79" s="2"/>
+      <c r="U79" s="19"/>
       <c r="V79" s="2"/>
-      <c r="W79" s="2"/>
+      <c r="W79" s="19"/>
     </row>
     <row r="80" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
@@ -4140,9 +4215,9 @@
       <c r="R80" s="6"/>
       <c r="S80" s="6"/>
       <c r="T80" s="7"/>
-      <c r="U80" s="6"/>
+      <c r="U80" s="18"/>
       <c r="V80" s="6"/>
-      <c r="W80" s="6"/>
+      <c r="W80" s="18"/>
     </row>
     <row r="81" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
@@ -4167,9 +4242,9 @@
       <c r="R81" s="2"/>
       <c r="S81" s="2"/>
       <c r="T81" s="3"/>
-      <c r="U81" s="2"/>
+      <c r="U81" s="19"/>
       <c r="V81" s="2"/>
-      <c r="W81" s="2"/>
+      <c r="W81" s="19"/>
     </row>
     <row r="82" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
@@ -4194,9 +4269,9 @@
       <c r="R82" s="6"/>
       <c r="S82" s="6"/>
       <c r="T82" s="7"/>
-      <c r="U82" s="6"/>
+      <c r="U82" s="18"/>
       <c r="V82" s="6"/>
-      <c r="W82" s="6"/>
+      <c r="W82" s="18"/>
     </row>
     <row r="83" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
@@ -4221,9 +4296,9 @@
       <c r="R83" s="2"/>
       <c r="S83" s="2"/>
       <c r="T83" s="3"/>
-      <c r="U83" s="2"/>
+      <c r="U83" s="19"/>
       <c r="V83" s="2"/>
-      <c r="W83" s="2"/>
+      <c r="W83" s="19"/>
     </row>
     <row r="84" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
@@ -4248,9 +4323,9 @@
       <c r="R84" s="6"/>
       <c r="S84" s="6"/>
       <c r="T84" s="7"/>
-      <c r="U84" s="6"/>
+      <c r="U84" s="18"/>
       <c r="V84" s="6"/>
-      <c r="W84" s="6"/>
+      <c r="W84" s="18"/>
     </row>
     <row r="85" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
@@ -4275,9 +4350,9 @@
       <c r="R85" s="2"/>
       <c r="S85" s="2"/>
       <c r="T85" s="3"/>
-      <c r="U85" s="2"/>
+      <c r="U85" s="19"/>
       <c r="V85" s="2"/>
-      <c r="W85" s="2"/>
+      <c r="W85" s="19"/>
     </row>
     <row r="86" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
@@ -4302,9 +4377,9 @@
       <c r="R86" s="6"/>
       <c r="S86" s="6"/>
       <c r="T86" s="7"/>
-      <c r="U86" s="6"/>
+      <c r="U86" s="18"/>
       <c r="V86" s="6"/>
-      <c r="W86" s="6"/>
+      <c r="W86" s="18"/>
     </row>
     <row r="87" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
@@ -4329,9 +4404,9 @@
       <c r="R87" s="2"/>
       <c r="S87" s="2"/>
       <c r="T87" s="3"/>
-      <c r="U87" s="2"/>
+      <c r="U87" s="19"/>
       <c r="V87" s="2"/>
-      <c r="W87" s="2"/>
+      <c r="W87" s="19"/>
     </row>
     <row r="88" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
@@ -4356,9 +4431,9 @@
       <c r="R88" s="6"/>
       <c r="S88" s="6"/>
       <c r="T88" s="7"/>
-      <c r="U88" s="6"/>
+      <c r="U88" s="18"/>
       <c r="V88" s="6"/>
-      <c r="W88" s="6"/>
+      <c r="W88" s="18"/>
     </row>
     <row r="89" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
@@ -4383,9 +4458,9 @@
       <c r="R89" s="2"/>
       <c r="S89" s="2"/>
       <c r="T89" s="3"/>
-      <c r="U89" s="2"/>
+      <c r="U89" s="19"/>
       <c r="V89" s="2"/>
-      <c r="W89" s="2"/>
+      <c r="W89" s="19"/>
     </row>
     <row r="90" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
@@ -4410,9 +4485,9 @@
       <c r="R90" s="6"/>
       <c r="S90" s="6"/>
       <c r="T90" s="7"/>
-      <c r="U90" s="6"/>
+      <c r="U90" s="18"/>
       <c r="V90" s="6"/>
-      <c r="W90" s="6"/>
+      <c r="W90" s="18"/>
     </row>
     <row r="91" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
@@ -4437,9 +4512,9 @@
       <c r="R91" s="2"/>
       <c r="S91" s="2"/>
       <c r="T91" s="3"/>
-      <c r="U91" s="2"/>
+      <c r="U91" s="19"/>
       <c r="V91" s="2"/>
-      <c r="W91" s="2"/>
+      <c r="W91" s="19"/>
     </row>
     <row r="92" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
@@ -4464,9 +4539,9 @@
       <c r="R92" s="6"/>
       <c r="S92" s="6"/>
       <c r="T92" s="7"/>
-      <c r="U92" s="6"/>
+      <c r="U92" s="18"/>
       <c r="V92" s="6"/>
-      <c r="W92" s="6"/>
+      <c r="W92" s="18"/>
     </row>
     <row r="93" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
@@ -4491,9 +4566,9 @@
       <c r="R93" s="2"/>
       <c r="S93" s="2"/>
       <c r="T93" s="3"/>
-      <c r="U93" s="2"/>
+      <c r="U93" s="19"/>
       <c r="V93" s="2"/>
-      <c r="W93" s="2"/>
+      <c r="W93" s="19"/>
     </row>
     <row r="94" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
@@ -4518,9 +4593,9 @@
       <c r="R94" s="6"/>
       <c r="S94" s="6"/>
       <c r="T94" s="7"/>
-      <c r="U94" s="6"/>
+      <c r="U94" s="18"/>
       <c r="V94" s="6"/>
-      <c r="W94" s="6"/>
+      <c r="W94" s="18"/>
     </row>
     <row r="95" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
@@ -4545,9 +4620,9 @@
       <c r="R95" s="2"/>
       <c r="S95" s="2"/>
       <c r="T95" s="3"/>
-      <c r="U95" s="2"/>
+      <c r="U95" s="19"/>
       <c r="V95" s="2"/>
-      <c r="W95" s="2"/>
+      <c r="W95" s="19"/>
     </row>
     <row r="96" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
@@ -4572,9 +4647,9 @@
       <c r="R96" s="6"/>
       <c r="S96" s="6"/>
       <c r="T96" s="7"/>
-      <c r="U96" s="6"/>
+      <c r="U96" s="18"/>
       <c r="V96" s="6"/>
-      <c r="W96" s="6"/>
+      <c r="W96" s="18"/>
     </row>
     <row r="97" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
@@ -4599,9 +4674,9 @@
       <c r="R97" s="2"/>
       <c r="S97" s="2"/>
       <c r="T97" s="3"/>
-      <c r="U97" s="2"/>
+      <c r="U97" s="19"/>
       <c r="V97" s="2"/>
-      <c r="W97" s="2"/>
+      <c r="W97" s="19"/>
     </row>
     <row r="98" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
@@ -4626,9 +4701,9 @@
       <c r="R98" s="6"/>
       <c r="S98" s="6"/>
       <c r="T98" s="7"/>
-      <c r="U98" s="6"/>
+      <c r="U98" s="18"/>
       <c r="V98" s="6"/>
-      <c r="W98" s="6"/>
+      <c r="W98" s="18"/>
     </row>
     <row r="99" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
@@ -4653,9 +4728,9 @@
       <c r="R99" s="2"/>
       <c r="S99" s="2"/>
       <c r="T99" s="3"/>
-      <c r="U99" s="2"/>
+      <c r="U99" s="19"/>
       <c r="V99" s="2"/>
-      <c r="W99" s="2"/>
+      <c r="W99" s="19"/>
     </row>
     <row r="100" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
@@ -4680,9 +4755,9 @@
       <c r="R100" s="6"/>
       <c r="S100" s="6"/>
       <c r="T100" s="7"/>
-      <c r="U100" s="6"/>
+      <c r="U100" s="18"/>
       <c r="V100" s="6"/>
-      <c r="W100" s="6"/>
+      <c r="W100" s="18"/>
     </row>
     <row r="101" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
@@ -4707,9 +4782,9 @@
       <c r="R101" s="2"/>
       <c r="S101" s="2"/>
       <c r="T101" s="3"/>
-      <c r="U101" s="2"/>
+      <c r="U101" s="19"/>
       <c r="V101" s="2"/>
-      <c r="W101" s="2"/>
+      <c r="W101" s="19"/>
     </row>
     <row r="102" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A102" s="6" t="s">
@@ -4734,13 +4809,13 @@
       <c r="R102" s="6"/>
       <c r="S102" s="6"/>
       <c r="T102" s="7"/>
-      <c r="U102" s="6"/>
+      <c r="U102" s="18"/>
       <c r="V102" s="6"/>
-      <c r="W102" s="6"/>
+      <c r="W102" s="18"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:W102">
-    <sortCondition descending="1" ref="K3:K102"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:W14">
+    <sortCondition descending="1" ref="K3:K14"/>
   </sortState>
   <mergeCells count="18">
     <mergeCell ref="A1:A2"/>
@@ -4839,23 +4914,23 @@
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="19" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="B1" s="19" t="s">
+    <row r="1" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="E1" s="19" t="s">
+      <c r="C1" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="E1" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="15" t="s">
         <v>116</v>
       </c>
     </row>
@@ -4866,17 +4941,17 @@
       <c r="B2" t="s">
         <v>139</v>
       </c>
-      <c r="C2" s="20">
+      <c r="C2" s="16">
         <v>1</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -4884,19 +4959,19 @@
         <v>138</v>
       </c>
       <c r="B3" t="s">
-        <v>163</v>
-      </c>
-      <c r="C3" s="20">
+        <v>161</v>
+      </c>
+      <c r="C3" s="16">
         <v>2</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -4904,49 +4979,49 @@
         <v>137</v>
       </c>
       <c r="B4" t="s">
-        <v>164</v>
-      </c>
-      <c r="C4" s="20">
+        <v>162</v>
+      </c>
+      <c r="C4" s="16">
         <v>3</v>
       </c>
       <c r="D4">
         <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B5" t="s">
-        <v>165</v>
-      </c>
-      <c r="C5" s="20">
+        <v>163</v>
+      </c>
+      <c r="C5" s="16">
         <v>4</v>
       </c>
       <c r="D5">
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B6" t="s">
         <v>140</v>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="16">
         <v>5</v>
       </c>
       <c r="D6">
@@ -4954,22 +5029,22 @@
       </c>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Governance Week 6 update
</commit_message>
<xml_diff>
--- a/IT Risk Register.xlsx
+++ b/IT Risk Register.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\salmo\Desktop\Tech\03 Projects\Enterprise Network Lab\03 Governance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD1DC5F-B2D1-45BF-9F35-4202CBAC1695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBF72125-A52C-4687-B53D-CA2BEE59F921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EE207035-1F51-4DCC-B353-2E8B956805B3}"/>
+    <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{EE207035-1F51-4DCC-B353-2E8B956805B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Operational Risk Register" sheetId="1" r:id="rId1"/>
@@ -294,7 +294,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="196">
   <si>
     <t>Risk Title</t>
   </si>
@@ -867,6 +867,21 @@
   </si>
   <si>
     <t>Develop a centralized application to automate and improve implementation of the change control policy</t>
+  </si>
+  <si>
+    <t>Implement device-specific administrative and privileged (enable) passwords as an interim containment measure. Restrict credential distribution to authorised personnel based on operational need, reducing unauthorized access and limiting exposure until formal identity-based access controls are implemented.</t>
+  </si>
+  <si>
+    <t>Relocate network devices to the most secure available offices within each floor, building, and campus. Restrict physical access by securing rooms with locked doors and implementing controlled key access under third-party supervision, requiring formal sign-out and return procedures. Re-route cabling as required to support relocation and ensure devices are not accessible from unsecured or public areas.</t>
+  </si>
+  <si>
+    <t>Deploy dedicated secure network infrastructure areas using locked racks within controlled-access rooms. Implement RFID-based access control with centralised management, environmental protections (fire suppression and climate control), and integrated monitoring systems to ensure all physical and administrative access is restricted, logged, and auditable.</t>
+  </si>
+  <si>
+    <t>Configure secure administrative access on all network devices by setting unique device-level and privileged (enable) passwords, removing default credentials, and restricting access to authorised personnel only.</t>
+  </si>
+  <si>
+    <t>Configure secure administrative access on all network devices by implementing unique device-level and privileged (enable) passwords, removing default credentials, and restricting access to authorised personnel.</t>
   </si>
 </sst>
 </file>
@@ -1210,10 +1225,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1222,32 +1261,8 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1632,9 +1647,9 @@
     <col min="12" max="12" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="67.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="59.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="46.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="48.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="63" style="4" customWidth="1"/>
+    <col min="16" max="16" width="59.85546875" style="4" customWidth="1"/>
+    <col min="17" max="17" width="58.5703125" style="4" customWidth="1"/>
     <col min="18" max="18" width="30" style="4" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="33.85546875" style="4" customWidth="1"/>
     <col min="20" max="20" width="51.140625" style="5" customWidth="1"/>
@@ -1645,72 +1660,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="F1" s="32" t="s">
+      <c r="F1" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="32" t="s">
+      <c r="G1" s="36"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="33"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="30" t="s">
+      <c r="J1" s="36"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="30" t="s">
+      <c r="M1" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="30" t="s">
+      <c r="N1" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="30" t="s">
+      <c r="O1" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="P1" s="30" t="s">
+      <c r="P1" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="Q1" s="30" t="s">
+      <c r="Q1" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="R1" s="30" t="s">
+      <c r="R1" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="S1" s="30" t="s">
+      <c r="S1" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="T1" s="32" t="s">
+      <c r="T1" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="U1" s="34"/>
-      <c r="V1" s="24" t="s">
+      <c r="U1" s="31"/>
+      <c r="V1" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="W1" s="26" t="s">
+      <c r="W1" s="34" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:23" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31"/>
-      <c r="B2" s="31"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="25"/>
+      <c r="A2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="29"/>
       <c r="F2" s="9" t="s">
         <v>1</v>
       </c>
@@ -1729,22 +1744,22 @@
       <c r="K2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="31"/>
-      <c r="S2" s="31"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="27"/>
       <c r="T2" s="12" t="s">
         <v>12</v>
       </c>
       <c r="U2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="V2" s="25"/>
-      <c r="W2" s="27"/>
+      <c r="V2" s="29"/>
+      <c r="W2" s="35"/>
     </row>
     <row r="3" spans="1:23" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
@@ -1807,7 +1822,7 @@
       <c r="T3" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="U3" s="35">
+      <c r="U3" s="24">
         <v>46132</v>
       </c>
       <c r="V3" s="13" t="s">
@@ -1863,7 +1878,7 @@
       <c r="O4" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="P4" s="36" t="s">
+      <c r="P4" s="25" t="s">
         <v>189</v>
       </c>
       <c r="Q4" s="6" t="s">
@@ -1959,7 +1974,7 @@
         <v>46133</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" ht="126" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>26</v>
       </c>
@@ -1986,23 +2001,47 @@
         <v>15</v>
       </c>
       <c r="I6" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J6" s="4">
         <v>5</v>
       </c>
       <c r="K6" s="4">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M6" s="4">
         <v>4</v>
       </c>
+      <c r="N6" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="O6" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="P6" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q6" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="R6" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="T6" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="U6" s="20">
+        <v>46147</v>
+      </c>
       <c r="V6" s="4" t="s">
         <v>154</v>
       </c>
       <c r="W6" s="20">
-        <v>46089</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4818,6 +4857,12 @@
     <sortCondition descending="1" ref="K3:K14"/>
   </sortState>
   <mergeCells count="18">
+    <mergeCell ref="V1:V2"/>
+    <mergeCell ref="W1:W2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="R1:R2"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="I1:K1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="E1:E2"/>
@@ -4830,12 +4875,6 @@
     <mergeCell ref="S1:S2"/>
     <mergeCell ref="L1:L2"/>
     <mergeCell ref="D1:D2"/>
-    <mergeCell ref="V1:V2"/>
-    <mergeCell ref="W1:W2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="R1:R2"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="I1:K1"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="L3:L1048576">

</xml_diff>